<commit_message>
Add energy consumption type field and split CAPEX/OPEX in the UI
Adds a ninth input, energyType (gas/electric/blended), validated and
recorded server-side but with no confirmed effect on the model yet -
Adaptavate hasn't defined that relationship, so it's a deliberate no-op
rather than an invented one. Input validation in prepare_inputs is now
table-driven (BOUNDS + a new ENUM_FIELDS registry in contract.py) so a
future field is a table entry, not a rewrite.

Also splits the dashboard's combined CAPEX/OPEX tile into two separate
metric cards, surfaced while manually verifying scenarios against the
live engine.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/Adaptavate-BBE-TEST-model.xlsx
+++ b/model/Adaptavate-BBE-TEST-model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Calculations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Internal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="in_feedstock_carbon">'Inputs'!$B$2</definedName>

</xml_diff>